<commit_message>
docs(sqap): versión 1.2 del plan con familias crítico y matriz alineada a Jenkins
- Tabla 4, Anexos B y C y jest.config.ts: familias (US-20 y consulta del
  padre de US-11) pasa a ser módulo crítico con 90 % de cobertura (M06).
- matrices-sqap, hoja Métricas: cada umbral apunta a su etapa del
  Jenkinsfile y no a ci.yml, deploy.yml o perf.yml, que no existen;
  M01 y M02 con el mismo momento que la Tabla 9.
- Tabla 24: pdfkit en vez de pdfmake, y ioredis.
- Anexo F y glosario: pendientes cerrados con D1 a D20, cliente piloto
  (Unidad Educativa Nazareno), aprobación de US-17 a US-20, monitor
  UptimeRobot y canales WhatsApp y Discord.

Refs: US-20
</commit_message>
<xml_diff>
--- a/docs/sqap/matrices-sqap.xlsx
+++ b/docs/sqap/matrices-sqap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="325">
   <si>
     <t xml:space="preserve">Métricas de calidad (Sección 5 del SQAP)</t>
   </si>
@@ -82,7 +82,7 @@
     <t xml:space="preserve">Suite calculo.casos.spec.ts</t>
   </si>
   <si>
-    <t xml:space="preserve">Cada PR y push</t>
+    <t xml:space="preserve">Cada build de Jenkins (PR y main)</t>
   </si>
   <si>
     <t xml:space="preserve">100 %</t>
@@ -94,7 +94,7 @@
     <t xml:space="preserve">Dev backend (Lujan)</t>
   </si>
   <si>
-    <t xml:space="preserve">ci.yml, job test-api: Jest termina con error si un caso falla</t>
+    <t xml:space="preserve">Jenkinsfile, etapa Pruebas › API: npm run -w api test:cov + junit; el build falla si un caso falla</t>
   </si>
   <si>
     <t xml:space="preserve">Completitud</t>
@@ -112,7 +112,7 @@
     <t xml:space="preserve">Staging con datos sintéticos</t>
   </si>
   <si>
-    <t xml:space="preserve">Cada merge a main y cada RC</t>
+    <t xml:space="preserve">Cada build de develop</t>
   </si>
   <si>
     <t xml:space="preserve">RNF-02</t>
@@ -121,7 +121,7 @@
     <t xml:space="preserve">Tester (Galvan)</t>
   </si>
   <si>
-    <t xml:space="preserve">deploy.yml, job e2e: npx cypress run</t>
+    <t xml:space="preserve">Jenkinsfile, etapa E2E (rama develop): npx cypress run</t>
   </si>
   <si>
     <t xml:space="preserve">Eficiencia de desempeño</t>
@@ -151,7 +151,7 @@
     <t xml:space="preserve">RNF-03</t>
   </si>
   <si>
-    <t xml:space="preserve">perf.yml: jq -e ".Total.pct2ResTime &lt;= 2000" perf/boletin/statistics.json</t>
+    <t xml:space="preserve">Jenkinsfile, etapa Rendimiento (etiquetas v*-rc.*): jq -e ".Total.pct2ResTime &lt;= 2000" perf/boletin/statistics.json</t>
   </si>
   <si>
     <t xml:space="preserve">Capacidad</t>
@@ -169,7 +169,7 @@
     <t xml:space="preserve">RNF-03, R05</t>
   </si>
   <si>
-    <t xml:space="preserve">perf.yml: jq -e ".Total.errorPct &lt; 1" en perf/boletin y perf/planilla</t>
+    <t xml:space="preserve">Jenkinsfile, etapa Rendimiento (etiquetas v*-rc.*): jq -e ".Total.errorPct &lt; 1" en perf/boletin y perf/planilla</t>
   </si>
   <si>
     <t xml:space="preserve">Mantenibilidad</t>
@@ -214,7 +214,7 @@
     <t xml:space="preserve">Jest coverageThreshold (P1, P2)</t>
   </si>
   <si>
-    <t xml:space="preserve">notas, calculo, auditoria, auth</t>
+    <t xml:space="preserve">notas, calculo, auditoria, auth, familias</t>
   </si>
   <si>
     <t xml:space="preserve">≥ 90 % por módulo</t>
@@ -271,7 +271,7 @@
     <t xml:space="preserve">RNF-04, R06</t>
   </si>
   <si>
-    <t xml:space="preserve">Quality Gate: Security Rating on New Code is worse than A; ci.yml job audit: npm audit --audit-level=high</t>
+    <t xml:space="preserve">Quality Gate: Security Rating on New Code is worse than A; Jenkinsfile, etapa Dependencias: npm audit --audit-level=high</t>
   </si>
   <si>
     <t xml:space="preserve">Integridad</t>
@@ -292,7 +292,7 @@
     <t xml:space="preserve">RNF-04</t>
   </si>
   <si>
-    <t xml:space="preserve">ci.yml, job test-api: npm run -w api test:e2e</t>
+    <t xml:space="preserve">Jenkinsfile, etapa Pruebas › API: suite autorizacion.e2e-spec.ts dentro de npm run -w api test:cov</t>
   </si>
   <si>
     <t xml:space="preserve">Usabilidad</t>
@@ -376,7 +376,7 @@
     <t xml:space="preserve">RNF-07</t>
   </si>
   <si>
-    <t xml:space="preserve">Monitor externo: intervalo 5 min</t>
+    <t xml:space="preserve">UptimeRobot: intervalo 5 min sobre /api/salud</t>
   </si>
   <si>
     <t xml:space="preserve">Recuperabilidad</t>
@@ -418,6 +418,9 @@
     <t xml:space="preserve">Suite auditoria.e2e-spec.ts</t>
   </si>
   <si>
+    <t xml:space="preserve">Jenkinsfile, etapa Pruebas › API: suite auditoria.e2e-spec.ts dentro de npm run -w api test:cov</t>
+  </si>
+  <si>
     <t xml:space="preserve">Analizabilidad</t>
   </si>
   <si>
@@ -436,7 +439,7 @@
     <t xml:space="preserve">Pre-commit y cada PR</t>
   </si>
   <si>
-    <t xml:space="preserve">ci.yml, job lint: eslint . --max-warnings=0; prettier --check .</t>
+    <t xml:space="preserve">Jenkinsfile, etapa Lint y hook pre-commit: eslint . --max-warnings=0; prettier --check .</t>
   </si>
   <si>
     <t xml:space="preserve">Matriz de riesgos de calidad (Sección 14 del SQAP)</t>
@@ -1965,7 +1968,7 @@
         <v>22</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>89</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1973,22 +1976,22 @@
         <v>49</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H19" s="5" t="s">
         <v>80</v>
@@ -2000,7 +2003,7 @@
         <v>58</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2089,58 +2092,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>3</v>
@@ -2157,27 +2160,27 @@
         <v>Alto</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>2</v>
@@ -2194,27 +2197,27 @@
         <v>Alto</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>2</v>
@@ -2231,27 +2234,27 @@
         <v>Alto</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>2</v>
@@ -2268,27 +2271,27 @@
         <v>Alto</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>3</v>
@@ -2305,27 +2308,27 @@
         <v>Alto</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
@@ -2342,27 +2345,27 @@
         <v>Alto</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>1</v>
@@ -2379,27 +2382,27 @@
         <v>Medio</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>3</v>
@@ -2416,27 +2419,27 @@
         <v>Alto</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>3</v>
@@ -2453,27 +2456,27 @@
         <v>Alto</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>2</v>
@@ -2490,27 +2493,27 @@
         <v>Medio</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -2527,24 +2530,24 @@
         <v>Medio</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>74</v>
@@ -2564,27 +2567,27 @@
         <v>Medio</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>2</v>
@@ -2601,27 +2604,27 @@
         <v>Alto</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>2</v>
@@ -2638,16 +2641,16 @@
         <v>Medio</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2788,112 +2791,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>255</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>254</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>255</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>253</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2941,506 +2944,506 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F5" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>276</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>277</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F7" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F9" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>292</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>291</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>292</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F14" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F15" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="H15" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F16" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F17" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="H17" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F18" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F19" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>306</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>305</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F20" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>316</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>271</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>274</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="F21" s="6" t="s">
+      <c r="H21" s="6" t="s">
         <v>274</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>316</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(sqap): Quality Gate "Sonar way" y M05, M07 y M08 en cada build de develop
SonarQube Cloud quedó conectado (T-030). Secciones 5 y 9, Anexo C,
matrices-sqap y metricas.md: el gate se llama "Sonar way" y se mide en
develop, la única rama que analiza el plan gratuito. Los umbrales no
cambian.

Refs: T-030
</commit_message>
<xml_diff>
--- a/docs/sqap/matrices-sqap.xlsx
+++ b/docs/sqap/matrices-sqap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="325">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="326">
   <si>
     <t xml:space="preserve">Métricas de calidad (Sección 5 del SQAP)</t>
   </si>
@@ -190,33 +190,33 @@
     <t xml:space="preserve">Código nuevo del PR</t>
   </si>
   <si>
+    <t xml:space="preserve">≥ 80 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RNF-05, R03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Responsable SQA (Galvan)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quality Gate: Coverage on New Code is less than 80.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">M06 · Cobertura de líneas de cada módulo crítico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">líneas cubiertas / líneas del módulo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jest coverageThreshold (P1, P2)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">notas, calculo, auditoria, auth, familias</t>
+  </si>
+  <si>
     <t xml:space="preserve">Cada PR</t>
   </si>
   <si>
-    <t xml:space="preserve">≥ 80 %</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RNF-05, R03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Responsable SQA (Galvan)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Quality Gate: Coverage on New Code is less than 80.0</t>
-  </si>
-  <si>
-    <t xml:space="preserve">M06 · Cobertura de líneas de cada módulo crítico</t>
-  </si>
-  <si>
-    <t xml:space="preserve">líneas cubiertas / líneas del módulo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jest coverageThreshold (P1, P2)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notas, calculo, auditoria, auth, familias</t>
-  </si>
-  <si>
     <t xml:space="preserve">≥ 90 % por módulo</t>
   </si>
   <si>
@@ -263,6 +263,9 @@
   </si>
   <si>
     <t xml:space="preserve">Código nuevo y package-lock.json</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cada build (SonarQube: develop)</t>
   </si>
   <si>
     <t xml:space="preserve">0</t>
@@ -1641,19 +1644,19 @@
         <v>54</v>
       </c>
       <c r="G9" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="H9" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="H9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="I9" s="5" t="s">
+      <c r="J9" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="J9" s="5" t="s">
+      <c r="K9" s="5" t="s">
         <v>58</v>
-      </c>
-      <c r="K9" s="5" t="s">
-        <v>59</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1664,19 +1667,19 @@
         <v>50</v>
       </c>
       <c r="C10" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="E10" s="5" t="s">
+      <c r="F10" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="F10" s="5" t="s">
+      <c r="G10" s="5" t="s">
         <v>63</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="H10" s="5" t="s">
         <v>64</v>
@@ -1685,7 +1688,7 @@
         <v>65</v>
       </c>
       <c r="J10" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K10" s="5" t="s">
         <v>66</v>
@@ -1711,7 +1714,7 @@
         <v>54</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>55</v>
+        <v>29</v>
       </c>
       <c r="H11" s="5" t="s">
         <v>71</v>
@@ -1720,7 +1723,7 @@
         <v>72</v>
       </c>
       <c r="J11" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K11" s="5" t="s">
         <v>73</v>
@@ -1746,19 +1749,19 @@
         <v>79</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>55</v>
+        <v>80</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I12" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="J12" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K12" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1766,174 +1769,174 @@
         <v>74</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="H13" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I13" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J13" s="5" t="s">
         <v>22</v>
       </c>
       <c r="K13" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="I14" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J14" s="5" t="s">
         <v>31</v>
       </c>
       <c r="K14" s="5" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I15" s="5" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J15" s="5" t="s">
         <v>31</v>
       </c>
       <c r="K15" s="5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="I16" s="5" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="J16" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K16" s="5" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I17" s="5" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J17" s="5" t="s">
         <v>22</v>
       </c>
       <c r="K17" s="5" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1941,34 +1944,34 @@
         <v>74</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="H18" s="5" t="s">
         <v>20</v>
       </c>
       <c r="I18" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J18" s="5" t="s">
         <v>22</v>
       </c>
       <c r="K18" s="5" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1976,34 +1979,34 @@
         <v>49</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="I19" s="5" t="s">
         <v>72</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K19" s="5" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2092,58 +2095,58 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="I4" s="4" t="s">
         <v>11</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>3</v>
@@ -2160,27 +2163,27 @@
         <v>Alto</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>2</v>
@@ -2197,27 +2200,27 @@
         <v>Alto</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>2</v>
@@ -2234,27 +2237,27 @@
         <v>Alto</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>2</v>
@@ -2271,27 +2274,27 @@
         <v>Alto</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="I8" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="K8" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="D9" s="6" t="n">
         <v>3</v>
@@ -2308,27 +2311,27 @@
         <v>Alto</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="I9" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D10" s="6" t="n">
         <v>2</v>
@@ -2345,27 +2348,27 @@
         <v>Alto</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="I10" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D11" s="6" t="n">
         <v>1</v>
@@ -2382,27 +2385,27 @@
         <v>Medio</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="I11" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="K11" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>3</v>
@@ -2419,27 +2422,27 @@
         <v>Alto</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="I12" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J12" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="K12" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="D13" s="6" t="n">
         <v>3</v>
@@ -2456,27 +2459,27 @@
         <v>Alto</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="I13" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J13" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K13" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>2</v>
@@ -2493,27 +2496,27 @@
         <v>Medio</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="I14" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J14" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K14" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D15" s="6" t="n">
         <v>1</v>
@@ -2530,24 +2533,24 @@
         <v>Medio</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="I15" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J15" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="K15" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C16" s="6" t="s">
         <v>74</v>
@@ -2567,27 +2570,27 @@
         <v>Medio</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="I16" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="K16" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="D17" s="6" t="n">
         <v>2</v>
@@ -2604,27 +2607,27 @@
         <v>Alto</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="I17" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="K17" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="D18" s="6" t="n">
         <v>2</v>
@@ -2641,16 +2644,16 @@
         <v>Medio</v>
       </c>
       <c r="H18" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="I18" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="K18" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2791,112 +2794,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>256</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>257</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>259</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>255</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>256</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>257</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>258</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>259</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>254</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2944,506 +2947,506 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F5" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H5" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>279</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="F6" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>277</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>278</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="F6" s="6" t="s">
+      <c r="H6" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H6" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F7" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G7" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F8" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H8" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H8" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F9" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G9" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H9" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F10" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H10" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G10" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H10" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
+        <v>293</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>294</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D12" s="6" t="s">
+        <v>295</v>
+      </c>
+      <c r="E12" s="6" t="s">
+        <v>296</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>292</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>293</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>294</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>295</v>
-      </c>
-      <c r="F12" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>291</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F14" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H14" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F15" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="H15" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G15" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="H15" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F16" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="H16" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="H16" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F17" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="H17" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="H17" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D18" s="6" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="E18" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F18" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="H18" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F19" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>307</v>
+      </c>
+      <c r="H19" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G19" s="6" t="s">
-        <v>306</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F20" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G20" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="H20" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G20" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
+        <v>319</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>272</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>273</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>320</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>275</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>276</v>
+      </c>
+      <c r="G21" s="6" t="s">
         <v>318</v>
       </c>
-      <c r="B21" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>319</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>274</v>
-      </c>
-      <c r="F21" s="6" t="s">
+      <c r="H21" s="6" t="s">
         <v>275</v>
-      </c>
-      <c r="G21" s="6" t="s">
-        <v>317</v>
-      </c>
-      <c r="H21" s="6" t="s">
-        <v>274</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs(sqap): revisión OWASP del Sprint 3, postmortem de CAL-001 y riesgo R15
Acta de la revisión contra el OWASP Top 10 (ZAP y revisión manual):
H1 y H2 corregidos, H3 (CAL-003) y H4 (CAL-004) abiertos, H5 aceptado.
Postmortem de CAL-001 (S1). CAL-001 y CAL-002 comparten causa: se
registra R15 en el SQAP y en matrices-sqap; helmet entra en la Tabla 24
y en Componentes de terceros.

Refs: CAL-001
</commit_message>
<xml_diff>
--- a/docs/sqap/matrices-sqap.xlsx
+++ b/docs/sqap/matrices-sqap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="475" uniqueCount="326">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="336">
   <si>
     <t xml:space="preserve">Métricas de calidad (Sección 5 del SQAP)</t>
   </si>
@@ -721,6 +721,21 @@
     <t xml:space="preserve">El cambio pasa al sprint siguiente o a la Release 2.</t>
   </si>
   <si>
+    <t xml:space="preserve">R15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Una automatización (pipeline, despliegue o respaldo) falla o no se ejecuta sin que nadie lo note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revisar cada día hábil el último build de develop y los runs de backup (postmortem CAL-001); UptimeRobot cada 5 min; la imagen comprueba sus dependencias al construirse</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Un build de develop o un run de backup en rojo más de 1 día hábil</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Se registra como defecto S2 y se corrige antes que cualquier tarea del sprint</t>
+  </si>
+  <si>
     <t xml:space="preserve">SLA de gestión de defectos (Sección 8 del SQAP)</t>
   </si>
   <si>
@@ -1001,6 +1016,21 @@
   </si>
   <si>
     <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">helmet</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.3.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabeceras de seguridad de la API (revisión OWASP del Sprint 3, H1, A05); la recomienda la documentación de NestJS; sin dependencias ni scripts de instalación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12/07/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30/10/2026</t>
   </si>
 </sst>
 </file>
@@ -2657,23 +2687,41 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6"/>
-      <c r="B19" s="6"/>
-      <c r="C19" s="6"/>
-      <c r="D19" s="6"/>
-      <c r="E19" s="6"/>
-      <c r="F19" s="6" t="str">
+      <c r="A19" s="6" t="s">
+        <v>232</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>233</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>174</v>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" s="6" t="n">
         <f aca="false">IF(OR(D19="",E19=""),"",D19*E19)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="G19" s="6" t="str">
         <f aca="false">IF(F19="","",IF(F19&gt;=6,"Alto",IF(F19&gt;=3,"Medio","Bajo")))</f>
-        <v/>
-      </c>
-      <c r="H19" s="6"/>
-      <c r="I19" s="6"/>
-      <c r="J19" s="6"/>
-      <c r="K19" s="6"/>
+        <v>Alto</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>234</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>169</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>235</v>
+      </c>
+      <c r="K19" s="6" t="s">
+        <v>236</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6"/>
@@ -2794,112 +2842,112 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="28.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="E8" s="6" t="s">
+        <v>265</v>
+      </c>
+      <c r="F8" s="6" t="s">
         <v>260</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>255</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2934,7 +2982,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
@@ -2947,506 +2995,532 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="H4" s="4" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
+        <v>283</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>278</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>273</v>
-      </c>
       <c r="D6" s="6" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
+        <v>285</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>286</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>280</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>281</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>276</v>
-      </c>
       <c r="G7" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
+        <v>287</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>288</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G8" s="6" t="s">
         <v>282</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>283</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="G8" s="6" t="s">
-        <v>277</v>
-      </c>
       <c r="H8" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>294</v>
+        <v>299</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D12" s="6" t="s">
-        <v>295</v>
+        <v>300</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H12" s="6" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="6" t="s">
-        <v>297</v>
+        <v>302</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>298</v>
+        <v>303</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D13" s="6" t="s">
-        <v>299</v>
+        <v>304</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>300</v>
+        <v>305</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H13" s="6" t="s">
-        <v>302</v>
+        <v>307</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>303</v>
+        <v>308</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>304</v>
+        <v>309</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G14" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>305</v>
+        <v>310</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D15" s="6" t="s">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F15" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="H15" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="6" t="s">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D16" s="6" t="s">
-        <v>309</v>
+        <v>314</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G16" s="6" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="H16" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="6" t="s">
-        <v>310</v>
+        <v>315</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="E17" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G17" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="6" t="s">
+        <v>317</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>277</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>318</v>
+      </c>
+      <c r="E18" s="6" t="s">
+        <v>280</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="B18" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>273</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>313</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>275</v>
-      </c>
-      <c r="F18" s="6" t="s">
-        <v>276</v>
-      </c>
-      <c r="G18" s="6" t="s">
-        <v>307</v>
-      </c>
       <c r="H18" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="6" t="s">
-        <v>314</v>
+        <v>319</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D19" s="6" t="s">
-        <v>315</v>
+        <v>320</v>
       </c>
       <c r="E19" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G19" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="H19" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="6" t="s">
-        <v>316</v>
+        <v>321</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D20" s="6" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="E20" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G20" s="6" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="H20" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="41.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>320</v>
+        <v>325</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F21" s="6" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
       <c r="H21" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="6" t="s">
-        <v>321</v>
+        <v>326</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>322</v>
+        <v>327</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>323</v>
+        <v>328</v>
       </c>
       <c r="D22" s="6" t="s">
-        <v>324</v>
+        <v>329</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="F22" s="6" t="s">
-        <v>325</v>
+        <v>330</v>
       </c>
       <c r="G22" s="6" t="s">
-        <v>307</v>
+        <v>312</v>
       </c>
       <c r="H22" s="6" t="s">
-        <v>275</v>
+        <v>280</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="6" t="s">
+        <v>331</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>332</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>278</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>333</v>
+      </c>
+      <c r="E23" s="6" t="s">
+        <v>334</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>281</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>282</v>
+      </c>
+      <c r="H23" s="6" t="s">
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>